<commit_message>
Adding Excel files & images & notes
</commit_message>
<xml_diff>
--- a/Excel/Book1.xlsx
+++ b/Excel/Book1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\j-l-data-science-data-analytics\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC5DFC43-0CC2-4843-84CD-5E390959E859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3A077DC-8411-43BD-972C-C2174FF0F84D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{F7F01B57-B888-4E05-A171-2C1A91DBF350}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="32">
   <si>
     <t>Employee Payroll</t>
   </si>
@@ -128,6 +128,9 @@
   <si>
     <t>Total Pay</t>
   </si>
+  <si>
+    <t>Jan Pay</t>
+  </si>
 </sst>
 </file>
 
@@ -135,7 +138,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="169" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -153,15 +156,51 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -169,20 +208,114 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top style="thin">
+        <color theme="2"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="16" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -498,46 +631,58 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A488FA1-4119-4E7F-B14C-64FC004B9D39}">
-  <dimension ref="A1:M25"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:AD25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="14.85546875" customWidth="1"/>
-    <col min="4" max="9" width="14.7109375" customWidth="1"/>
-    <col min="10" max="10" width="19" customWidth="1"/>
-    <col min="11" max="11" width="14.5703125" customWidth="1"/>
-    <col min="12" max="12" width="18.140625" customWidth="1"/>
-    <col min="13" max="13" width="17" customWidth="1"/>
+    <col min="4" max="8" width="14.7109375" customWidth="1"/>
+    <col min="9" max="13" width="19" customWidth="1"/>
+    <col min="14" max="18" width="14.5703125" customWidth="1"/>
+    <col min="19" max="23" width="18.140625" customWidth="1"/>
+    <col min="24" max="24" width="17" customWidth="1"/>
+    <col min="25" max="25" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="18.5703125" customWidth="1"/>
+    <col min="31" max="31" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1"/>
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4"/>
       <c r="C1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
         <v>4</v>
       </c>
-      <c r="J2" t="s">
+      <c r="I2" t="s">
         <v>28</v>
       </c>
-      <c r="K2" t="s">
+      <c r="N2" t="s">
         <v>5</v>
       </c>
-      <c r="L2" t="s">
+      <c r="S2" t="s">
         <v>29</v>
       </c>
-      <c r="M2" t="s">
+      <c r="X2" t="s">
         <v>30</v>
       </c>
+      <c r="AD2" t="s">
+        <v>31</v>
+      </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -547,648 +692,2512 @@
       <c r="C3" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="5">
         <v>46023</v>
       </c>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
+      <c r="E3" s="5">
+        <f>D3+7</f>
+        <v>46030</v>
+      </c>
+      <c r="F3" s="5">
+        <f t="shared" ref="F3:H3" si="0">E3+7</f>
+        <v>46037</v>
+      </c>
+      <c r="G3" s="5">
+        <f t="shared" si="0"/>
+        <v>46044</v>
+      </c>
+      <c r="H3" s="5">
+        <f t="shared" si="0"/>
+        <v>46051</v>
+      </c>
+      <c r="I3" s="7">
+        <v>46023</v>
+      </c>
+      <c r="J3" s="7">
+        <f>I3+7</f>
+        <v>46030</v>
+      </c>
+      <c r="K3" s="7">
+        <f t="shared" ref="K3:M3" si="1">J3+7</f>
+        <v>46037</v>
+      </c>
+      <c r="L3" s="7">
+        <f t="shared" si="1"/>
+        <v>46044</v>
+      </c>
+      <c r="M3" s="7">
+        <f t="shared" si="1"/>
+        <v>46051</v>
+      </c>
+      <c r="N3" s="9">
+        <v>46023</v>
+      </c>
+      <c r="O3" s="9">
+        <f>N3+7</f>
+        <v>46030</v>
+      </c>
+      <c r="P3" s="9">
+        <f t="shared" ref="P3:R3" si="2">O3+7</f>
+        <v>46037</v>
+      </c>
+      <c r="Q3" s="9">
+        <f t="shared" si="2"/>
+        <v>46044</v>
+      </c>
+      <c r="R3" s="9">
+        <f t="shared" si="2"/>
+        <v>46051</v>
+      </c>
+      <c r="S3" s="11">
+        <v>46023</v>
+      </c>
+      <c r="T3" s="11">
+        <f>S3+7</f>
+        <v>46030</v>
+      </c>
+      <c r="U3" s="11">
+        <f t="shared" ref="U3:W3" si="3">T3+7</f>
+        <v>46037</v>
+      </c>
+      <c r="V3" s="13">
+        <f t="shared" si="3"/>
+        <v>46044</v>
+      </c>
+      <c r="W3" s="14">
+        <f t="shared" si="3"/>
+        <v>46051</v>
+      </c>
+      <c r="X3" s="18">
+        <v>46023</v>
+      </c>
+      <c r="Y3" s="18">
+        <f>X3+7</f>
+        <v>46030</v>
+      </c>
+      <c r="Z3" s="18">
+        <f t="shared" ref="Z3:AB3" si="4">Y3+7</f>
+        <v>46037</v>
+      </c>
+      <c r="AA3" s="18">
+        <f t="shared" si="4"/>
+        <v>46044</v>
+      </c>
+      <c r="AB3" s="18">
+        <f t="shared" si="4"/>
+        <v>46051</v>
+      </c>
+      <c r="AC3" s="17"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="1">
         <v>100</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="6">
         <v>40</v>
       </c>
-      <c r="J4">
+      <c r="E4" s="6">
+        <f ca="1">RANDBETWEEN(10, 90)</f>
+        <v>13</v>
+      </c>
+      <c r="F4" s="6">
+        <f t="shared" ref="F4:H4" ca="1" si="5">RANDBETWEEN(10, 90)</f>
+        <v>71</v>
+      </c>
+      <c r="G4" s="6">
+        <f t="shared" ca="1" si="5"/>
+        <v>24</v>
+      </c>
+      <c r="H4" s="6">
+        <f t="shared" ca="1" si="5"/>
+        <v>49</v>
+      </c>
+      <c r="I4" s="8">
         <f>IF(D4&gt;50,D4-50,0)</f>
         <v>0</v>
       </c>
-      <c r="K4" s="4">
-        <f>C4*D4</f>
+      <c r="J4" s="8">
+        <f ca="1">IF(E4&gt;50,E4-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K4" s="8">
+        <f ca="1">IF(F4&gt;50,F4-50,0)</f>
+        <v>21</v>
+      </c>
+      <c r="L4" s="8">
+        <f ca="1">IF(G4&gt;50,G4-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" s="8">
+        <f ca="1">IF(H4&gt;50,H4-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N4" s="10">
+        <f>$C4*D4</f>
         <v>4000</v>
       </c>
-      <c r="L4" s="4">
-        <f>0.5*C4*J4</f>
-        <v>0</v>
-      </c>
-      <c r="M4" s="4">
-        <f>K4+L4</f>
+      <c r="O4" s="10">
+        <f ca="1">$C4*E4</f>
+        <v>1300</v>
+      </c>
+      <c r="P4" s="10">
+        <f t="shared" ref="P4:R19" ca="1" si="6">$C4*F4</f>
+        <v>7100</v>
+      </c>
+      <c r="Q4" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>2400</v>
+      </c>
+      <c r="R4" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>4900</v>
+      </c>
+      <c r="S4" s="12">
+        <f>0.5*$C4*I4</f>
+        <v>0</v>
+      </c>
+      <c r="T4" s="12">
+        <f ca="1">0.5*$C4*J4</f>
+        <v>0</v>
+      </c>
+      <c r="U4" s="12">
+        <f t="shared" ref="U4:W19" ca="1" si="7">0.5*$C4*K4</f>
+        <v>1050</v>
+      </c>
+      <c r="V4" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="W4" s="15">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="X4" s="19">
+        <f>N4+S4</f>
         <v>4000</v>
       </c>
+      <c r="Y4" s="19">
+        <f t="shared" ref="Y4:AB19" ca="1" si="8">O4+T4</f>
+        <v>1300</v>
+      </c>
+      <c r="Z4" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>8150</v>
+      </c>
+      <c r="AA4" s="19">
+        <f ca="1">Q4+V4</f>
+        <v>2400</v>
+      </c>
+      <c r="AB4" s="19">
+        <f ca="1">R4+W4</f>
+        <v>4900</v>
+      </c>
+      <c r="AC4" s="17"/>
+      <c r="AD4" s="2">
+        <f ca="1">SUM(X4:AB4)</f>
+        <v>20750</v>
+      </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="1">
         <v>150</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="6">
         <v>40.5</v>
       </c>
-      <c r="J5">
+      <c r="E5" s="6">
+        <f t="shared" ref="E5:H20" ca="1" si="9">RANDBETWEEN(10, 90)</f>
+        <v>54</v>
+      </c>
+      <c r="F5" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>20</v>
+      </c>
+      <c r="G5" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>39</v>
+      </c>
+      <c r="H5" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>85</v>
+      </c>
+      <c r="I5" s="8">
         <f>IF(D5&gt;50,D5-50,0)</f>
         <v>0</v>
       </c>
-      <c r="K5" s="4">
-        <f t="shared" ref="K5:K23" si="0">C5*D5</f>
+      <c r="J5" s="8">
+        <f ca="1">IF(E5&gt;50,E5-50,0)</f>
+        <v>4</v>
+      </c>
+      <c r="K5" s="8">
+        <f ca="1">IF(F5&gt;50,F5-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="8">
+        <f ca="1">IF(G5&gt;50,G5-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="8">
+        <f ca="1">IF(H5&gt;50,H5-50,0)</f>
+        <v>35</v>
+      </c>
+      <c r="N5" s="10">
+        <f t="shared" ref="N5:N20" si="10">$C5*D5</f>
         <v>6075</v>
       </c>
-      <c r="L5" s="4">
-        <f t="shared" ref="L5:L20" si="1">0.5*C5*J5</f>
-        <v>0</v>
-      </c>
-      <c r="M5" s="4">
-        <f t="shared" ref="M5:M20" si="2">K5+L5</f>
+      <c r="O5" s="10">
+        <f t="shared" ref="O5:O20" ca="1" si="11">$C5*E5</f>
+        <v>8100</v>
+      </c>
+      <c r="P5" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>3000</v>
+      </c>
+      <c r="Q5" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>5850</v>
+      </c>
+      <c r="R5" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>12750</v>
+      </c>
+      <c r="S5" s="12">
+        <f t="shared" ref="S5:T20" si="12">0.5*$C5*I5</f>
+        <v>0</v>
+      </c>
+      <c r="T5" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>300</v>
+      </c>
+      <c r="U5" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="V5" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="W5" s="16">
+        <f t="shared" ca="1" si="7"/>
+        <v>2625</v>
+      </c>
+      <c r="X5" s="19">
+        <f>N5+S5</f>
         <v>6075</v>
       </c>
+      <c r="Y5" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>8400</v>
+      </c>
+      <c r="Z5" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>3000</v>
+      </c>
+      <c r="AA5" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>5850</v>
+      </c>
+      <c r="AB5" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>15375</v>
+      </c>
+      <c r="AC5" s="17"/>
+      <c r="AD5" s="2">
+        <f t="shared" ref="AD5:AD20" ca="1" si="13">SUM(X5:AB5)</f>
+        <v>38700</v>
+      </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="1">
         <v>200</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="6">
         <v>45</v>
       </c>
-      <c r="J6">
+      <c r="E6" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>19</v>
+      </c>
+      <c r="F6" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>87</v>
+      </c>
+      <c r="G6" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>38</v>
+      </c>
+      <c r="H6" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>78</v>
+      </c>
+      <c r="I6" s="8">
         <f>IF(D6&gt;50,D6-50,0)</f>
         <v>0</v>
       </c>
-      <c r="K6" s="4">
-        <f t="shared" si="0"/>
+      <c r="J6" s="8">
+        <f ca="1">IF(E6&gt;50,E6-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="8">
+        <f ca="1">IF(F6&gt;50,F6-50,0)</f>
+        <v>37</v>
+      </c>
+      <c r="L6" s="8">
+        <f ca="1">IF(G6&gt;50,G6-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M6" s="8">
+        <f ca="1">IF(H6&gt;50,H6-50,0)</f>
+        <v>28</v>
+      </c>
+      <c r="N6" s="10">
+        <f t="shared" si="10"/>
         <v>9000</v>
       </c>
-      <c r="L6" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="M6" s="4">
-        <f t="shared" si="2"/>
+      <c r="O6" s="10">
+        <f t="shared" ca="1" si="11"/>
+        <v>3800</v>
+      </c>
+      <c r="P6" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>17400</v>
+      </c>
+      <c r="Q6" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>7600</v>
+      </c>
+      <c r="R6" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>15600</v>
+      </c>
+      <c r="S6" s="12">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="T6" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="U6" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>3700</v>
+      </c>
+      <c r="V6" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="W6" s="16">
+        <f t="shared" ca="1" si="7"/>
+        <v>2800</v>
+      </c>
+      <c r="X6" s="19">
+        <f>N6+S6</f>
         <v>9000</v>
       </c>
+      <c r="Y6" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>3800</v>
+      </c>
+      <c r="Z6" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>21100</v>
+      </c>
+      <c r="AA6" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>7600</v>
+      </c>
+      <c r="AB6" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>18400</v>
+      </c>
+      <c r="AC6" s="17"/>
+      <c r="AD6" s="2">
+        <f t="shared" ca="1" si="13"/>
+        <v>59900</v>
+      </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="1">
         <v>250</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="6">
         <v>45.5</v>
       </c>
-      <c r="J7">
+      <c r="E7" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>67</v>
+      </c>
+      <c r="F7" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>19</v>
+      </c>
+      <c r="G7" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>73</v>
+      </c>
+      <c r="H7" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>29</v>
+      </c>
+      <c r="I7" s="8">
         <f>IF(D7&gt;50,D7-50,0)</f>
         <v>0</v>
       </c>
-      <c r="K7" s="4">
-        <f t="shared" si="0"/>
+      <c r="J7" s="8">
+        <f ca="1">IF(E7&gt;50,E7-50,0)</f>
+        <v>17</v>
+      </c>
+      <c r="K7" s="8">
+        <f ca="1">IF(F7&gt;50,F7-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="8">
+        <f ca="1">IF(G7&gt;50,G7-50,0)</f>
+        <v>23</v>
+      </c>
+      <c r="M7" s="8">
+        <f ca="1">IF(H7&gt;50,H7-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N7" s="10">
+        <f t="shared" si="10"/>
         <v>11375</v>
       </c>
-      <c r="L7" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="M7" s="4">
-        <f t="shared" si="2"/>
+      <c r="O7" s="10">
+        <f t="shared" ca="1" si="11"/>
+        <v>16750</v>
+      </c>
+      <c r="P7" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>4750</v>
+      </c>
+      <c r="Q7" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>18250</v>
+      </c>
+      <c r="R7" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>7250</v>
+      </c>
+      <c r="S7" s="12">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="T7" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>2125</v>
+      </c>
+      <c r="U7" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="V7" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>2875</v>
+      </c>
+      <c r="W7" s="16">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="X7" s="19">
+        <f>N7+S7</f>
         <v>11375</v>
       </c>
+      <c r="Y7" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>18875</v>
+      </c>
+      <c r="Z7" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>4750</v>
+      </c>
+      <c r="AA7" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>21125</v>
+      </c>
+      <c r="AB7" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>7250</v>
+      </c>
+      <c r="AC7" s="17"/>
+      <c r="AD7" s="2">
+        <f t="shared" ca="1" si="13"/>
+        <v>63375</v>
+      </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
       <c r="B8" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="1">
         <v>300</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="6">
         <v>50</v>
       </c>
-      <c r="J8">
+      <c r="E8" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>69</v>
+      </c>
+      <c r="F8" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>28</v>
+      </c>
+      <c r="G8" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>86</v>
+      </c>
+      <c r="H8" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>86</v>
+      </c>
+      <c r="I8" s="8">
         <f>IF(D8&gt;50,D8-50,0)</f>
         <v>0</v>
       </c>
-      <c r="K8" s="4">
-        <f t="shared" si="0"/>
+      <c r="J8" s="8">
+        <f ca="1">IF(E8&gt;50,E8-50,0)</f>
+        <v>19</v>
+      </c>
+      <c r="K8" s="8">
+        <f ca="1">IF(F8&gt;50,F8-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L8" s="8">
+        <f ca="1">IF(G8&gt;50,G8-50,0)</f>
+        <v>36</v>
+      </c>
+      <c r="M8" s="8">
+        <f ca="1">IF(H8&gt;50,H8-50,0)</f>
+        <v>36</v>
+      </c>
+      <c r="N8" s="10">
+        <f t="shared" si="10"/>
         <v>15000</v>
       </c>
-      <c r="L8" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="M8" s="4">
-        <f t="shared" si="2"/>
+      <c r="O8" s="10">
+        <f t="shared" ca="1" si="11"/>
+        <v>20700</v>
+      </c>
+      <c r="P8" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>8400</v>
+      </c>
+      <c r="Q8" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>25800</v>
+      </c>
+      <c r="R8" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>25800</v>
+      </c>
+      <c r="S8" s="12">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="T8" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>2850</v>
+      </c>
+      <c r="U8" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="V8" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>5400</v>
+      </c>
+      <c r="W8" s="16">
+        <f t="shared" ca="1" si="7"/>
+        <v>5400</v>
+      </c>
+      <c r="X8" s="19">
+        <f>N8+S8</f>
         <v>15000</v>
       </c>
+      <c r="Y8" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>23550</v>
+      </c>
+      <c r="Z8" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>8400</v>
+      </c>
+      <c r="AA8" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>31200</v>
+      </c>
+      <c r="AB8" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>31200</v>
+      </c>
+      <c r="AC8" s="17"/>
+      <c r="AD8" s="2">
+        <f t="shared" ca="1" si="13"/>
+        <v>109350</v>
+      </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="1">
         <v>350</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="6">
         <v>50.5</v>
       </c>
-      <c r="J9">
+      <c r="E9" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>90</v>
+      </c>
+      <c r="F9" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>30</v>
+      </c>
+      <c r="G9" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>14</v>
+      </c>
+      <c r="H9" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>70</v>
+      </c>
+      <c r="I9" s="8">
         <f>IF(D9&gt;50,D9-50,0)</f>
         <v>0.5</v>
       </c>
-      <c r="K9" s="4">
-        <f t="shared" si="0"/>
+      <c r="J9" s="8">
+        <f ca="1">IF(E9&gt;50,E9-50,0)</f>
+        <v>40</v>
+      </c>
+      <c r="K9" s="8">
+        <f ca="1">IF(F9&gt;50,F9-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L9" s="8">
+        <f ca="1">IF(G9&gt;50,G9-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M9" s="8">
+        <f ca="1">IF(H9&gt;50,H9-50,0)</f>
+        <v>20</v>
+      </c>
+      <c r="N9" s="10">
+        <f t="shared" si="10"/>
         <v>17675</v>
       </c>
-      <c r="L9" s="4">
-        <f t="shared" si="1"/>
+      <c r="O9" s="10">
+        <f t="shared" ca="1" si="11"/>
+        <v>31500</v>
+      </c>
+      <c r="P9" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>10500</v>
+      </c>
+      <c r="Q9" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>4900</v>
+      </c>
+      <c r="R9" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>24500</v>
+      </c>
+      <c r="S9" s="12">
+        <f t="shared" si="12"/>
         <v>87.5</v>
       </c>
-      <c r="M9" s="4">
-        <f t="shared" si="2"/>
+      <c r="T9" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>7000</v>
+      </c>
+      <c r="U9" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="V9" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="W9" s="16">
+        <f t="shared" ca="1" si="7"/>
+        <v>3500</v>
+      </c>
+      <c r="X9" s="19">
+        <f>N9+S9</f>
         <v>17762.5</v>
       </c>
+      <c r="Y9" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>38500</v>
+      </c>
+      <c r="Z9" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>10500</v>
+      </c>
+      <c r="AA9" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>4900</v>
+      </c>
+      <c r="AB9" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>28000</v>
+      </c>
+      <c r="AC9" s="17"/>
+      <c r="AD9" s="2">
+        <f t="shared" ca="1" si="13"/>
+        <v>99662.5</v>
+      </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
       <c r="B10" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="1">
         <v>400</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="6">
         <v>55</v>
       </c>
-      <c r="J10">
+      <c r="E10" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>54</v>
+      </c>
+      <c r="F10" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>51</v>
+      </c>
+      <c r="G10" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>69</v>
+      </c>
+      <c r="H10" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>23</v>
+      </c>
+      <c r="I10" s="8">
         <f>IF(D10&gt;50,D10-50,0)</f>
         <v>5</v>
       </c>
-      <c r="K10" s="4">
-        <f t="shared" si="0"/>
+      <c r="J10" s="8">
+        <f ca="1">IF(E10&gt;50,E10-50,0)</f>
+        <v>4</v>
+      </c>
+      <c r="K10" s="8">
+        <f ca="1">IF(F10&gt;50,F10-50,0)</f>
+        <v>1</v>
+      </c>
+      <c r="L10" s="8">
+        <f ca="1">IF(G10&gt;50,G10-50,0)</f>
+        <v>19</v>
+      </c>
+      <c r="M10" s="8">
+        <f ca="1">IF(H10&gt;50,H10-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N10" s="10">
+        <f t="shared" si="10"/>
         <v>22000</v>
       </c>
-      <c r="L10" s="4">
-        <f t="shared" si="1"/>
+      <c r="O10" s="10">
+        <f t="shared" ca="1" si="11"/>
+        <v>21600</v>
+      </c>
+      <c r="P10" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>20400</v>
+      </c>
+      <c r="Q10" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>27600</v>
+      </c>
+      <c r="R10" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>9200</v>
+      </c>
+      <c r="S10" s="12">
+        <f t="shared" si="12"/>
         <v>1000</v>
       </c>
-      <c r="M10" s="4">
-        <f t="shared" si="2"/>
+      <c r="T10" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>800</v>
+      </c>
+      <c r="U10" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>200</v>
+      </c>
+      <c r="V10" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>3800</v>
+      </c>
+      <c r="W10" s="16">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="X10" s="19">
+        <f>N10+S10</f>
         <v>23000</v>
       </c>
+      <c r="Y10" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>22400</v>
+      </c>
+      <c r="Z10" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>20600</v>
+      </c>
+      <c r="AA10" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>31400</v>
+      </c>
+      <c r="AB10" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>9200</v>
+      </c>
+      <c r="AC10" s="17"/>
+      <c r="AD10" s="2">
+        <f t="shared" ca="1" si="13"/>
+        <v>106600</v>
+      </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>13</v>
       </c>
       <c r="B11" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="1">
         <v>450</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="6">
         <v>55.5</v>
       </c>
-      <c r="J11">
+      <c r="E11" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>16</v>
+      </c>
+      <c r="F11" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>42</v>
+      </c>
+      <c r="G11" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>23</v>
+      </c>
+      <c r="H11" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>41</v>
+      </c>
+      <c r="I11" s="8">
         <f>IF(D11&gt;50,D11-50,0)</f>
         <v>5.5</v>
       </c>
-      <c r="K11" s="4">
-        <f t="shared" si="0"/>
+      <c r="J11" s="8">
+        <f ca="1">IF(E11&gt;50,E11-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="8">
+        <f ca="1">IF(F11&gt;50,F11-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L11" s="8">
+        <f ca="1">IF(G11&gt;50,G11-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M11" s="8">
+        <f ca="1">IF(H11&gt;50,H11-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N11" s="10">
+        <f t="shared" si="10"/>
         <v>24975</v>
       </c>
-      <c r="L11" s="4">
-        <f t="shared" si="1"/>
+      <c r="O11" s="10">
+        <f t="shared" ca="1" si="11"/>
+        <v>7200</v>
+      </c>
+      <c r="P11" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>18900</v>
+      </c>
+      <c r="Q11" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>10350</v>
+      </c>
+      <c r="R11" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>18450</v>
+      </c>
+      <c r="S11" s="12">
+        <f t="shared" si="12"/>
         <v>1237.5</v>
       </c>
-      <c r="M11" s="4">
-        <f t="shared" si="2"/>
+      <c r="T11" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="U11" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="V11" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="W11" s="16">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="X11" s="19">
+        <f>N11+S11</f>
         <v>26212.5</v>
       </c>
+      <c r="Y11" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>7200</v>
+      </c>
+      <c r="Z11" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>18900</v>
+      </c>
+      <c r="AA11" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>10350</v>
+      </c>
+      <c r="AB11" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>18450</v>
+      </c>
+      <c r="AC11" s="17"/>
+      <c r="AD11" s="2">
+        <f t="shared" ca="1" si="13"/>
+        <v>81112.5</v>
+      </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>14</v>
       </c>
       <c r="B12" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="1">
         <v>500</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="6">
         <v>60</v>
       </c>
-      <c r="J12">
+      <c r="E12" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>16</v>
+      </c>
+      <c r="F12" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>15</v>
+      </c>
+      <c r="G12" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>25</v>
+      </c>
+      <c r="H12" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>37</v>
+      </c>
+      <c r="I12" s="8">
         <f>IF(D12&gt;50,D12-50,0)</f>
         <v>10</v>
       </c>
-      <c r="K12" s="4">
-        <f t="shared" si="0"/>
+      <c r="J12" s="8">
+        <f ca="1">IF(E12&gt;50,E12-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K12" s="8">
+        <f ca="1">IF(F12&gt;50,F12-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L12" s="8">
+        <f ca="1">IF(G12&gt;50,G12-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M12" s="8">
+        <f ca="1">IF(H12&gt;50,H12-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N12" s="10">
+        <f t="shared" si="10"/>
         <v>30000</v>
       </c>
-      <c r="L12" s="4">
-        <f t="shared" si="1"/>
+      <c r="O12" s="10">
+        <f t="shared" ca="1" si="11"/>
+        <v>8000</v>
+      </c>
+      <c r="P12" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>7500</v>
+      </c>
+      <c r="Q12" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>12500</v>
+      </c>
+      <c r="R12" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>18500</v>
+      </c>
+      <c r="S12" s="12">
+        <f t="shared" si="12"/>
         <v>2500</v>
       </c>
-      <c r="M12" s="4">
-        <f t="shared" si="2"/>
+      <c r="T12" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="U12" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="V12" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="W12" s="16">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="X12" s="19">
+        <f>N12+S12</f>
         <v>32500</v>
       </c>
+      <c r="Y12" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>8000</v>
+      </c>
+      <c r="Z12" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>7500</v>
+      </c>
+      <c r="AA12" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>12500</v>
+      </c>
+      <c r="AB12" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>18500</v>
+      </c>
+      <c r="AC12" s="17"/>
+      <c r="AD12" s="2">
+        <f t="shared" ca="1" si="13"/>
+        <v>79000</v>
+      </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>15</v>
       </c>
       <c r="B13" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="1">
         <v>550</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="6">
         <v>60.5</v>
       </c>
-      <c r="J13">
+      <c r="E13" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>37</v>
+      </c>
+      <c r="F13" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>59</v>
+      </c>
+      <c r="G13" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>41</v>
+      </c>
+      <c r="H13" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>59</v>
+      </c>
+      <c r="I13" s="8">
         <f>IF(D13&gt;50,D13-50,0)</f>
         <v>10.5</v>
       </c>
-      <c r="K13" s="4">
-        <f t="shared" si="0"/>
+      <c r="J13" s="8">
+        <f ca="1">IF(E13&gt;50,E13-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="8">
+        <f ca="1">IF(F13&gt;50,F13-50,0)</f>
+        <v>9</v>
+      </c>
+      <c r="L13" s="8">
+        <f ca="1">IF(G13&gt;50,G13-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M13" s="8">
+        <f ca="1">IF(H13&gt;50,H13-50,0)</f>
+        <v>9</v>
+      </c>
+      <c r="N13" s="10">
+        <f t="shared" si="10"/>
         <v>33275</v>
       </c>
-      <c r="L13" s="4">
-        <f t="shared" si="1"/>
+      <c r="O13" s="10">
+        <f t="shared" ca="1" si="11"/>
+        <v>20350</v>
+      </c>
+      <c r="P13" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>32450</v>
+      </c>
+      <c r="Q13" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>22550</v>
+      </c>
+      <c r="R13" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>32450</v>
+      </c>
+      <c r="S13" s="12">
+        <f t="shared" si="12"/>
         <v>2887.5</v>
       </c>
-      <c r="M13" s="4">
-        <f t="shared" si="2"/>
+      <c r="T13" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="U13" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>2475</v>
+      </c>
+      <c r="V13" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="W13" s="16">
+        <f t="shared" ca="1" si="7"/>
+        <v>2475</v>
+      </c>
+      <c r="X13" s="19">
+        <f>N13+S13</f>
         <v>36162.5</v>
       </c>
+      <c r="Y13" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>20350</v>
+      </c>
+      <c r="Z13" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>34925</v>
+      </c>
+      <c r="AA13" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>22550</v>
+      </c>
+      <c r="AB13" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>34925</v>
+      </c>
+      <c r="AC13" s="17"/>
+      <c r="AD13" s="2">
+        <f t="shared" ca="1" si="13"/>
+        <v>148912.5</v>
+      </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>16</v>
       </c>
       <c r="B14" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="1">
         <v>600</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="6">
         <v>70</v>
       </c>
-      <c r="J14">
+      <c r="E14" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>19</v>
+      </c>
+      <c r="F14" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>83</v>
+      </c>
+      <c r="G14" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>27</v>
+      </c>
+      <c r="H14" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>52</v>
+      </c>
+      <c r="I14" s="8">
         <f>IF(D14&gt;50,D14-50,0)</f>
         <v>20</v>
       </c>
-      <c r="K14" s="4">
-        <f t="shared" si="0"/>
+      <c r="J14" s="8">
+        <f ca="1">IF(E14&gt;50,E14-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K14" s="8">
+        <f ca="1">IF(F14&gt;50,F14-50,0)</f>
+        <v>33</v>
+      </c>
+      <c r="L14" s="8">
+        <f ca="1">IF(G14&gt;50,G14-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M14" s="8">
+        <f ca="1">IF(H14&gt;50,H14-50,0)</f>
+        <v>2</v>
+      </c>
+      <c r="N14" s="10">
+        <f t="shared" si="10"/>
         <v>42000</v>
       </c>
-      <c r="L14" s="4">
-        <f t="shared" si="1"/>
+      <c r="O14" s="10">
+        <f t="shared" ca="1" si="11"/>
+        <v>11400</v>
+      </c>
+      <c r="P14" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>49800</v>
+      </c>
+      <c r="Q14" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>16200</v>
+      </c>
+      <c r="R14" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>31200</v>
+      </c>
+      <c r="S14" s="12">
+        <f t="shared" si="12"/>
         <v>6000</v>
       </c>
-      <c r="M14" s="4">
-        <f t="shared" si="2"/>
+      <c r="T14" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="U14" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>9900</v>
+      </c>
+      <c r="V14" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="W14" s="16">
+        <f t="shared" ca="1" si="7"/>
+        <v>600</v>
+      </c>
+      <c r="X14" s="19">
+        <f>N14+S14</f>
         <v>48000</v>
       </c>
+      <c r="Y14" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>11400</v>
+      </c>
+      <c r="Z14" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>59700</v>
+      </c>
+      <c r="AA14" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>16200</v>
+      </c>
+      <c r="AB14" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>31800</v>
+      </c>
+      <c r="AC14" s="17"/>
+      <c r="AD14" s="2">
+        <f t="shared" ca="1" si="13"/>
+        <v>167100</v>
+      </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
       <c r="B15" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="3">
+      <c r="C15" s="1">
         <v>650</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="6">
         <v>70.5</v>
       </c>
-      <c r="J15">
+      <c r="E15" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>62</v>
+      </c>
+      <c r="F15" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>21</v>
+      </c>
+      <c r="G15" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>73</v>
+      </c>
+      <c r="H15" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>73</v>
+      </c>
+      <c r="I15" s="8">
         <f>IF(D15&gt;50,D15-50,0)</f>
         <v>20.5</v>
       </c>
-      <c r="K15" s="4">
-        <f t="shared" si="0"/>
+      <c r="J15" s="8">
+        <f ca="1">IF(E15&gt;50,E15-50,0)</f>
+        <v>12</v>
+      </c>
+      <c r="K15" s="8">
+        <f ca="1">IF(F15&gt;50,F15-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L15" s="8">
+        <f ca="1">IF(G15&gt;50,G15-50,0)</f>
+        <v>23</v>
+      </c>
+      <c r="M15" s="8">
+        <f ca="1">IF(H15&gt;50,H15-50,0)</f>
+        <v>23</v>
+      </c>
+      <c r="N15" s="10">
+        <f t="shared" si="10"/>
         <v>45825</v>
       </c>
-      <c r="L15" s="4">
-        <f t="shared" si="1"/>
+      <c r="O15" s="10">
+        <f t="shared" ca="1" si="11"/>
+        <v>40300</v>
+      </c>
+      <c r="P15" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>13650</v>
+      </c>
+      <c r="Q15" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>47450</v>
+      </c>
+      <c r="R15" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>47450</v>
+      </c>
+      <c r="S15" s="12">
+        <f t="shared" si="12"/>
         <v>6662.5</v>
       </c>
-      <c r="M15" s="4">
-        <f t="shared" si="2"/>
+      <c r="T15" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>3900</v>
+      </c>
+      <c r="U15" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="V15" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>7475</v>
+      </c>
+      <c r="W15" s="16">
+        <f t="shared" ca="1" si="7"/>
+        <v>7475</v>
+      </c>
+      <c r="X15" s="19">
+        <f>N15+S15</f>
         <v>52487.5</v>
       </c>
+      <c r="Y15" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>44200</v>
+      </c>
+      <c r="Z15" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>13650</v>
+      </c>
+      <c r="AA15" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>54925</v>
+      </c>
+      <c r="AB15" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>54925</v>
+      </c>
+      <c r="AC15" s="17"/>
+      <c r="AD15" s="2">
+        <f t="shared" ca="1" si="13"/>
+        <v>220187.5</v>
+      </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>18</v>
       </c>
       <c r="B16" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C16" s="1">
         <v>700</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="6">
         <v>80</v>
       </c>
-      <c r="J16">
+      <c r="E16" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>55</v>
+      </c>
+      <c r="F16" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>11</v>
+      </c>
+      <c r="G16" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>48</v>
+      </c>
+      <c r="H16" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>31</v>
+      </c>
+      <c r="I16" s="8">
         <f>IF(D16&gt;50,D16-50,0)</f>
         <v>30</v>
       </c>
-      <c r="K16" s="4">
-        <f t="shared" si="0"/>
+      <c r="J16" s="8">
+        <f ca="1">IF(E16&gt;50,E16-50,0)</f>
+        <v>5</v>
+      </c>
+      <c r="K16" s="8">
+        <f ca="1">IF(F16&gt;50,F16-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L16" s="8">
+        <f ca="1">IF(G16&gt;50,G16-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M16" s="8">
+        <f ca="1">IF(H16&gt;50,H16-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N16" s="10">
+        <f t="shared" si="10"/>
         <v>56000</v>
       </c>
-      <c r="L16" s="4">
-        <f t="shared" si="1"/>
+      <c r="O16" s="10">
+        <f t="shared" ca="1" si="11"/>
+        <v>38500</v>
+      </c>
+      <c r="P16" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>7700</v>
+      </c>
+      <c r="Q16" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>33600</v>
+      </c>
+      <c r="R16" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>21700</v>
+      </c>
+      <c r="S16" s="12">
+        <f t="shared" si="12"/>
         <v>10500</v>
       </c>
-      <c r="M16" s="4">
-        <f t="shared" si="2"/>
+      <c r="T16" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>1750</v>
+      </c>
+      <c r="U16" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="V16" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="W16" s="16">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="X16" s="19">
+        <f>N16+S16</f>
         <v>66500</v>
       </c>
+      <c r="Y16" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>40250</v>
+      </c>
+      <c r="Z16" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>7700</v>
+      </c>
+      <c r="AA16" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>33600</v>
+      </c>
+      <c r="AB16" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>21700</v>
+      </c>
+      <c r="AC16" s="17"/>
+      <c r="AD16" s="2">
+        <f t="shared" ca="1" si="13"/>
+        <v>169750</v>
+      </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>19</v>
       </c>
       <c r="B17" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="3">
+      <c r="C17" s="1">
         <v>750</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="6">
         <v>80.5</v>
       </c>
-      <c r="J17">
+      <c r="E17" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>90</v>
+      </c>
+      <c r="F17" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>51</v>
+      </c>
+      <c r="G17" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>51</v>
+      </c>
+      <c r="H17" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>28</v>
+      </c>
+      <c r="I17" s="8">
         <f>IF(D17&gt;50,D17-50,0)</f>
         <v>30.5</v>
       </c>
-      <c r="K17" s="4">
-        <f t="shared" si="0"/>
+      <c r="J17" s="8">
+        <f ca="1">IF(E17&gt;50,E17-50,0)</f>
+        <v>40</v>
+      </c>
+      <c r="K17" s="8">
+        <f ca="1">IF(F17&gt;50,F17-50,0)</f>
+        <v>1</v>
+      </c>
+      <c r="L17" s="8">
+        <f ca="1">IF(G17&gt;50,G17-50,0)</f>
+        <v>1</v>
+      </c>
+      <c r="M17" s="8">
+        <f ca="1">IF(H17&gt;50,H17-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N17" s="10">
+        <f t="shared" si="10"/>
         <v>60375</v>
       </c>
-      <c r="L17" s="4">
-        <f t="shared" si="1"/>
+      <c r="O17" s="10">
+        <f t="shared" ca="1" si="11"/>
+        <v>67500</v>
+      </c>
+      <c r="P17" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>38250</v>
+      </c>
+      <c r="Q17" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>38250</v>
+      </c>
+      <c r="R17" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>21000</v>
+      </c>
+      <c r="S17" s="12">
+        <f t="shared" si="12"/>
         <v>11437.5</v>
       </c>
-      <c r="M17" s="4">
-        <f t="shared" si="2"/>
+      <c r="T17" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>15000</v>
+      </c>
+      <c r="U17" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>375</v>
+      </c>
+      <c r="V17" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>375</v>
+      </c>
+      <c r="W17" s="16">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="X17" s="19">
+        <f>N17+S17</f>
         <v>71812.5</v>
       </c>
+      <c r="Y17" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>82500</v>
+      </c>
+      <c r="Z17" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>38625</v>
+      </c>
+      <c r="AA17" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>38625</v>
+      </c>
+      <c r="AB17" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>21000</v>
+      </c>
+      <c r="AC17" s="17"/>
+      <c r="AD17" s="2">
+        <f t="shared" ca="1" si="13"/>
+        <v>252562.5</v>
+      </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>20</v>
       </c>
       <c r="B18" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C18" s="1">
         <v>850</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="6">
         <v>85</v>
       </c>
-      <c r="J18">
+      <c r="E18" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>32</v>
+      </c>
+      <c r="F18" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>51</v>
+      </c>
+      <c r="G18" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>51</v>
+      </c>
+      <c r="H18" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>84</v>
+      </c>
+      <c r="I18" s="8">
         <f>IF(D18&gt;50,D18-50,0)</f>
         <v>35</v>
       </c>
-      <c r="K18" s="4">
-        <f t="shared" si="0"/>
+      <c r="J18" s="8">
+        <f ca="1">IF(E18&gt;50,E18-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K18" s="8">
+        <f ca="1">IF(F18&gt;50,F18-50,0)</f>
+        <v>1</v>
+      </c>
+      <c r="L18" s="8">
+        <f ca="1">IF(G18&gt;50,G18-50,0)</f>
+        <v>1</v>
+      </c>
+      <c r="M18" s="8">
+        <f ca="1">IF(H18&gt;50,H18-50,0)</f>
+        <v>34</v>
+      </c>
+      <c r="N18" s="10">
+        <f t="shared" si="10"/>
         <v>72250</v>
       </c>
-      <c r="L18" s="4">
-        <f t="shared" si="1"/>
+      <c r="O18" s="10">
+        <f t="shared" ca="1" si="11"/>
+        <v>27200</v>
+      </c>
+      <c r="P18" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>43350</v>
+      </c>
+      <c r="Q18" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>43350</v>
+      </c>
+      <c r="R18" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>71400</v>
+      </c>
+      <c r="S18" s="12">
+        <f t="shared" si="12"/>
         <v>14875</v>
       </c>
-      <c r="M18" s="4">
-        <f t="shared" si="2"/>
+      <c r="T18" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="U18" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>425</v>
+      </c>
+      <c r="V18" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>425</v>
+      </c>
+      <c r="W18" s="16">
+        <f t="shared" ca="1" si="7"/>
+        <v>14450</v>
+      </c>
+      <c r="X18" s="19">
+        <f>N18+S18</f>
         <v>87125</v>
       </c>
+      <c r="Y18" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>27200</v>
+      </c>
+      <c r="Z18" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>43775</v>
+      </c>
+      <c r="AA18" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>43775</v>
+      </c>
+      <c r="AB18" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>85850</v>
+      </c>
+      <c r="AC18" s="17"/>
+      <c r="AD18" s="2">
+        <f t="shared" ca="1" si="13"/>
+        <v>287725</v>
+      </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>21</v>
       </c>
       <c r="B19" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="3">
+      <c r="C19" s="1">
         <v>900</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="6">
         <v>85.5</v>
       </c>
-      <c r="J19">
+      <c r="E19" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>46</v>
+      </c>
+      <c r="F19" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>39</v>
+      </c>
+      <c r="G19" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>32</v>
+      </c>
+      <c r="H19" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>79</v>
+      </c>
+      <c r="I19" s="8">
         <f>IF(D19&gt;50,D19-50,0)</f>
         <v>35.5</v>
       </c>
-      <c r="K19" s="4">
-        <f t="shared" si="0"/>
+      <c r="J19" s="8">
+        <f ca="1">IF(E19&gt;50,E19-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K19" s="8">
+        <f ca="1">IF(F19&gt;50,F19-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L19" s="8">
+        <f ca="1">IF(G19&gt;50,G19-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M19" s="8">
+        <f ca="1">IF(H19&gt;50,H19-50,0)</f>
+        <v>29</v>
+      </c>
+      <c r="N19" s="10">
+        <f t="shared" si="10"/>
         <v>76950</v>
       </c>
-      <c r="L19" s="4">
-        <f t="shared" si="1"/>
+      <c r="O19" s="10">
+        <f t="shared" ca="1" si="11"/>
+        <v>41400</v>
+      </c>
+      <c r="P19" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>35100</v>
+      </c>
+      <c r="Q19" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>28800</v>
+      </c>
+      <c r="R19" s="10">
+        <f t="shared" ca="1" si="6"/>
+        <v>71100</v>
+      </c>
+      <c r="S19" s="12">
+        <f t="shared" si="12"/>
         <v>15975</v>
       </c>
-      <c r="M19" s="4">
-        <f t="shared" si="2"/>
+      <c r="T19" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="U19" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="V19" s="12">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="W19" s="16">
+        <f t="shared" ca="1" si="7"/>
+        <v>13050</v>
+      </c>
+      <c r="X19" s="19">
+        <f>N19+S19</f>
         <v>92925</v>
       </c>
+      <c r="Y19" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>41400</v>
+      </c>
+      <c r="Z19" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>35100</v>
+      </c>
+      <c r="AA19" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>28800</v>
+      </c>
+      <c r="AB19" s="19">
+        <f t="shared" ca="1" si="8"/>
+        <v>84150</v>
+      </c>
+      <c r="AC19" s="17"/>
+      <c r="AD19" s="2">
+        <f t="shared" ca="1" si="13"/>
+        <v>282375</v>
+      </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>22</v>
       </c>
       <c r="B20" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C20" s="1">
         <v>1000</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="6">
         <v>90</v>
       </c>
-      <c r="J20">
+      <c r="E20" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>73</v>
+      </c>
+      <c r="F20" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>67</v>
+      </c>
+      <c r="G20" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>55</v>
+      </c>
+      <c r="H20" s="6">
+        <f t="shared" ca="1" si="9"/>
+        <v>18</v>
+      </c>
+      <c r="I20" s="8">
         <f>IF(D20&gt;50,D20-50,0)</f>
         <v>40</v>
       </c>
-      <c r="K20" s="4">
-        <f t="shared" si="0"/>
+      <c r="J20" s="8">
+        <f ca="1">IF(E20&gt;50,E20-50,0)</f>
+        <v>23</v>
+      </c>
+      <c r="K20" s="8">
+        <f ca="1">IF(F20&gt;50,F20-50,0)</f>
+        <v>17</v>
+      </c>
+      <c r="L20" s="8">
+        <f ca="1">IF(G20&gt;50,G20-50,0)</f>
+        <v>5</v>
+      </c>
+      <c r="M20" s="8">
+        <f ca="1">IF(H20&gt;50,H20-50,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N20" s="10">
+        <f t="shared" si="10"/>
         <v>90000</v>
       </c>
-      <c r="L20" s="4">
-        <f t="shared" si="1"/>
+      <c r="O20" s="10">
+        <f t="shared" ca="1" si="11"/>
+        <v>73000</v>
+      </c>
+      <c r="P20" s="10">
+        <f t="shared" ref="P20" ca="1" si="14">$C20*F20</f>
+        <v>67000</v>
+      </c>
+      <c r="Q20" s="10">
+        <f t="shared" ref="Q20" ca="1" si="15">$C20*G20</f>
+        <v>55000</v>
+      </c>
+      <c r="R20" s="10">
+        <f t="shared" ref="R20" ca="1" si="16">$C20*H20</f>
+        <v>18000</v>
+      </c>
+      <c r="S20" s="12">
+        <f t="shared" si="12"/>
         <v>20000</v>
       </c>
-      <c r="M20" s="4">
-        <f t="shared" si="2"/>
+      <c r="T20" s="12">
+        <f t="shared" ca="1" si="12"/>
+        <v>11500</v>
+      </c>
+      <c r="U20" s="12">
+        <f t="shared" ref="U20" ca="1" si="17">0.5*$C20*K20</f>
+        <v>8500</v>
+      </c>
+      <c r="V20" s="12">
+        <f t="shared" ref="V20" ca="1" si="18">0.5*$C20*L20</f>
+        <v>2500</v>
+      </c>
+      <c r="W20" s="16">
+        <f t="shared" ref="W20" ca="1" si="19">0.5*$C20*M20</f>
+        <v>0</v>
+      </c>
+      <c r="X20" s="19">
+        <f>N20+S20</f>
         <v>110000</v>
       </c>
+      <c r="Y20" s="19">
+        <f t="shared" ref="Y20:AB20" ca="1" si="20">O20+T20</f>
+        <v>84500</v>
+      </c>
+      <c r="Z20" s="19">
+        <f t="shared" ca="1" si="20"/>
+        <v>75500</v>
+      </c>
+      <c r="AA20" s="19">
+        <f t="shared" ca="1" si="20"/>
+        <v>57500</v>
+      </c>
+      <c r="AB20" s="19">
+        <f t="shared" ca="1" si="20"/>
+        <v>18000</v>
+      </c>
+      <c r="AC20" s="17"/>
+      <c r="AD20" s="2">
+        <f t="shared" ca="1" si="13"/>
+        <v>345500</v>
+      </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="4">
+      <c r="C22" s="2">
         <f>MAX(C4:C20)</f>
         <v>1000</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22" s="3">
         <f>MAX(D4:D20)</f>
         <v>90</v>
       </c>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="4">
-        <f>MAX(K4:K20)</f>
+      <c r="E22" s="2">
+        <f t="shared" ref="E22:AB22" ca="1" si="21">MAX(E4:E20)</f>
+        <v>90</v>
+      </c>
+      <c r="F22" s="3">
+        <f t="shared" ca="1" si="21"/>
+        <v>87</v>
+      </c>
+      <c r="G22" s="2">
+        <f t="shared" ca="1" si="21"/>
+        <v>86</v>
+      </c>
+      <c r="H22" s="3">
+        <f t="shared" ca="1" si="21"/>
+        <v>86</v>
+      </c>
+      <c r="I22" s="2">
+        <f t="shared" si="21"/>
+        <v>40</v>
+      </c>
+      <c r="J22" s="3">
+        <f t="shared" ca="1" si="21"/>
+        <v>40</v>
+      </c>
+      <c r="K22" s="2">
+        <f t="shared" ca="1" si="21"/>
+        <v>37</v>
+      </c>
+      <c r="L22" s="3">
+        <f t="shared" ca="1" si="21"/>
+        <v>36</v>
+      </c>
+      <c r="M22" s="2">
+        <f t="shared" ca="1" si="21"/>
+        <v>36</v>
+      </c>
+      <c r="N22" s="1">
+        <f t="shared" si="21"/>
         <v>90000</v>
       </c>
-      <c r="L22" s="4">
-        <f t="shared" ref="L22:M22" si="3">MAX(L4:L20)</f>
+      <c r="O22" s="2">
+        <f t="shared" ca="1" si="21"/>
+        <v>73000</v>
+      </c>
+      <c r="P22" s="3">
+        <f t="shared" ca="1" si="21"/>
+        <v>67000</v>
+      </c>
+      <c r="Q22" s="2">
+        <f t="shared" ca="1" si="21"/>
+        <v>55000</v>
+      </c>
+      <c r="R22" s="3">
+        <f t="shared" ca="1" si="21"/>
+        <v>71400</v>
+      </c>
+      <c r="S22" s="2">
+        <f t="shared" si="21"/>
         <v>20000</v>
       </c>
-      <c r="M22" s="4">
-        <f t="shared" si="3"/>
+      <c r="T22" s="3">
+        <f t="shared" ca="1" si="21"/>
+        <v>15000</v>
+      </c>
+      <c r="U22" s="2">
+        <f t="shared" ca="1" si="21"/>
+        <v>9900</v>
+      </c>
+      <c r="V22" s="1">
+        <f t="shared" ca="1" si="21"/>
+        <v>7475</v>
+      </c>
+      <c r="W22" s="2">
+        <f t="shared" ca="1" si="21"/>
+        <v>14450</v>
+      </c>
+      <c r="X22" s="3">
+        <f t="shared" si="21"/>
         <v>110000</v>
       </c>
+      <c r="Y22" s="2">
+        <f t="shared" ca="1" si="21"/>
+        <v>84500</v>
+      </c>
+      <c r="Z22" s="1">
+        <f t="shared" ca="1" si="21"/>
+        <v>75500</v>
+      </c>
+      <c r="AA22" s="2">
+        <f t="shared" ca="1" si="21"/>
+        <v>57500</v>
+      </c>
+      <c r="AB22" s="1">
+        <f t="shared" ca="1" si="21"/>
+        <v>85850</v>
+      </c>
+      <c r="AC22" s="1"/>
+      <c r="AD22" s="1">
+        <f t="shared" ref="AC22:AD22" ca="1" si="22">MAX(AD4:AD20)</f>
+        <v>345500</v>
+      </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="4">
+      <c r="C23" s="2">
         <f>MIN(C4:C20)</f>
         <v>100</v>
       </c>
-      <c r="D23" s="5">
+      <c r="D23" s="3">
         <f>MIN(D4:D20)</f>
         <v>40</v>
       </c>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="4">
-        <f>MIN(K4:K20)</f>
+      <c r="E23" s="2">
+        <f t="shared" ref="E23:AB23" ca="1" si="23">MIN(E4:E20)</f>
+        <v>13</v>
+      </c>
+      <c r="F23" s="3">
+        <f t="shared" ca="1" si="23"/>
+        <v>11</v>
+      </c>
+      <c r="G23" s="2">
+        <f t="shared" ca="1" si="23"/>
+        <v>14</v>
+      </c>
+      <c r="H23" s="3">
+        <f t="shared" ca="1" si="23"/>
+        <v>18</v>
+      </c>
+      <c r="I23" s="2">
+        <f t="shared" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="J23" s="3">
+        <f t="shared" ca="1" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="K23" s="2">
+        <f t="shared" ca="1" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="L23" s="3">
+        <f t="shared" ca="1" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="M23" s="2">
+        <f t="shared" ca="1" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="N23" s="1">
+        <f t="shared" si="23"/>
         <v>4000</v>
       </c>
-      <c r="L23" s="4">
-        <f t="shared" ref="L23:M23" si="4">MIN(L4:L20)</f>
-        <v>0</v>
-      </c>
-      <c r="M23" s="4">
-        <f t="shared" si="4"/>
+      <c r="O23" s="2">
+        <f t="shared" ca="1" si="23"/>
+        <v>1300</v>
+      </c>
+      <c r="P23" s="3">
+        <f t="shared" ca="1" si="23"/>
+        <v>3000</v>
+      </c>
+      <c r="Q23" s="2">
+        <f t="shared" ca="1" si="23"/>
+        <v>2400</v>
+      </c>
+      <c r="R23" s="3">
+        <f t="shared" ca="1" si="23"/>
+        <v>4900</v>
+      </c>
+      <c r="S23" s="2">
+        <f t="shared" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="T23" s="3">
+        <f t="shared" ca="1" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="U23" s="2">
+        <f t="shared" ca="1" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="V23" s="1">
+        <f t="shared" ca="1" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="W23" s="2">
+        <f t="shared" ca="1" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="X23" s="3">
+        <f t="shared" si="23"/>
         <v>4000</v>
       </c>
+      <c r="Y23" s="2">
+        <f t="shared" ca="1" si="23"/>
+        <v>1300</v>
+      </c>
+      <c r="Z23" s="1">
+        <f t="shared" ca="1" si="23"/>
+        <v>3000</v>
+      </c>
+      <c r="AA23" s="2">
+        <f t="shared" ca="1" si="23"/>
+        <v>2400</v>
+      </c>
+      <c r="AB23" s="1">
+        <f t="shared" ca="1" si="23"/>
+        <v>4900</v>
+      </c>
+      <c r="AC23" s="1"/>
+      <c r="AD23" s="1">
+        <f t="shared" ref="AC23:AD23" ca="1" si="24">MIN(AD4:AD20)</f>
+        <v>20750</v>
+      </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>25</v>
       </c>
-      <c r="C24" s="4">
+      <c r="C24" s="2">
         <f>AVERAGE(C4:C20)</f>
         <v>511.76470588235293</v>
       </c>
-      <c r="D24" s="5">
+      <c r="D24" s="3">
         <f>AVERAGE(D4:D20)</f>
         <v>62.588235294117645</v>
       </c>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="4">
-        <f>AVERAGE(K4:K20)</f>
+      <c r="E24" s="2">
+        <f t="shared" ref="E24:AB24" ca="1" si="25">AVERAGE(E4:E20)</f>
+        <v>47.764705882352942</v>
+      </c>
+      <c r="F24" s="3">
+        <f t="shared" ca="1" si="25"/>
+        <v>43.823529411764703</v>
+      </c>
+      <c r="G24" s="2">
+        <f t="shared" ca="1" si="25"/>
+        <v>45.235294117647058</v>
+      </c>
+      <c r="H24" s="3">
+        <f t="shared" ca="1" si="25"/>
+        <v>54.235294117647058</v>
+      </c>
+      <c r="I24" s="2">
+        <f t="shared" si="25"/>
+        <v>14.294117647058824</v>
+      </c>
+      <c r="J24" s="3">
+        <f t="shared" ca="1" si="25"/>
+        <v>9.6470588235294112</v>
+      </c>
+      <c r="K24" s="2">
+        <f t="shared" ca="1" si="25"/>
+        <v>7.0588235294117645</v>
+      </c>
+      <c r="L24" s="3">
+        <f t="shared" ca="1" si="25"/>
+        <v>6.3529411764705879</v>
+      </c>
+      <c r="M24" s="2">
+        <f t="shared" ca="1" si="25"/>
+        <v>12.705882352941176</v>
+      </c>
+      <c r="N24" s="1">
+        <f t="shared" si="25"/>
         <v>36280.882352941175</v>
       </c>
-      <c r="L24" s="4">
-        <f t="shared" ref="L24:M24" si="5">AVERAGE(L4:L20)</f>
+      <c r="O24" s="2">
+        <f t="shared" ca="1" si="25"/>
+        <v>25800</v>
+      </c>
+      <c r="P24" s="3">
+        <f t="shared" ca="1" si="25"/>
+        <v>22661.764705882353</v>
+      </c>
+      <c r="Q24" s="2">
+        <f t="shared" ca="1" si="25"/>
+        <v>23555.882352941175</v>
+      </c>
+      <c r="R24" s="3">
+        <f t="shared" ca="1" si="25"/>
+        <v>26544.117647058825</v>
+      </c>
+      <c r="S24" s="2">
+        <f t="shared" si="25"/>
         <v>5480.1470588235297</v>
       </c>
-      <c r="M24" s="4">
-        <f t="shared" si="5"/>
+      <c r="T24" s="3">
+        <f t="shared" ca="1" si="25"/>
+        <v>2660.294117647059</v>
+      </c>
+      <c r="U24" s="2">
+        <f t="shared" ca="1" si="25"/>
+        <v>1566.1764705882354</v>
+      </c>
+      <c r="V24" s="1">
+        <f t="shared" ca="1" si="25"/>
+        <v>1344.1176470588234</v>
+      </c>
+      <c r="W24" s="2">
+        <f t="shared" ca="1" si="25"/>
+        <v>3080.8823529411766</v>
+      </c>
+      <c r="X24" s="3">
+        <f t="shared" si="25"/>
         <v>41761.029411764706</v>
       </c>
+      <c r="Y24" s="2">
+        <f t="shared" ca="1" si="25"/>
+        <v>28460.294117647059</v>
+      </c>
+      <c r="Z24" s="1">
+        <f t="shared" ca="1" si="25"/>
+        <v>24227.941176470587</v>
+      </c>
+      <c r="AA24" s="2">
+        <f t="shared" ca="1" si="25"/>
+        <v>24900</v>
+      </c>
+      <c r="AB24" s="1">
+        <f t="shared" ca="1" si="25"/>
+        <v>29625</v>
+      </c>
+      <c r="AC24" s="1"/>
+      <c r="AD24" s="1">
+        <f t="shared" ref="AC24:AD24" ca="1" si="26">AVERAGE(AD4:AD20)</f>
+        <v>148974.26470588235</v>
+      </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>26</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C25" s="2">
         <f>SUM(C4:C20)</f>
         <v>8700</v>
       </c>
-      <c r="D25" s="5">
+      <c r="D25" s="3">
         <f>SUM(D4:D20)</f>
         <v>1064</v>
       </c>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
-      <c r="J25" s="5"/>
-      <c r="K25" s="4">
-        <f>SUM(K4:K20)</f>
+      <c r="E25" s="2">
+        <f t="shared" ref="E25:AB25" ca="1" si="27">SUM(E4:E20)</f>
+        <v>812</v>
+      </c>
+      <c r="F25" s="3">
+        <f t="shared" ca="1" si="27"/>
+        <v>745</v>
+      </c>
+      <c r="G25" s="2">
+        <f t="shared" ca="1" si="27"/>
+        <v>769</v>
+      </c>
+      <c r="H25" s="3">
+        <f t="shared" ca="1" si="27"/>
+        <v>922</v>
+      </c>
+      <c r="I25" s="2">
+        <f t="shared" si="27"/>
+        <v>243</v>
+      </c>
+      <c r="J25" s="3">
+        <f t="shared" ca="1" si="27"/>
+        <v>164</v>
+      </c>
+      <c r="K25" s="2">
+        <f t="shared" ca="1" si="27"/>
+        <v>120</v>
+      </c>
+      <c r="L25" s="3">
+        <f t="shared" ca="1" si="27"/>
+        <v>108</v>
+      </c>
+      <c r="M25" s="2">
+        <f t="shared" ca="1" si="27"/>
+        <v>216</v>
+      </c>
+      <c r="N25" s="1">
+        <f t="shared" si="27"/>
         <v>616775</v>
       </c>
-      <c r="L25" s="4">
-        <f t="shared" ref="L25:M25" si="6">SUM(L4:L20)</f>
+      <c r="O25" s="2">
+        <f t="shared" ca="1" si="27"/>
+        <v>438600</v>
+      </c>
+      <c r="P25" s="3">
+        <f t="shared" ca="1" si="27"/>
+        <v>385250</v>
+      </c>
+      <c r="Q25" s="2">
+        <f t="shared" ca="1" si="27"/>
+        <v>400450</v>
+      </c>
+      <c r="R25" s="3">
+        <f t="shared" ca="1" si="27"/>
+        <v>451250</v>
+      </c>
+      <c r="S25" s="2">
+        <f t="shared" si="27"/>
         <v>93162.5</v>
       </c>
-      <c r="M25" s="4">
-        <f t="shared" si="6"/>
+      <c r="T25" s="3">
+        <f t="shared" ca="1" si="27"/>
+        <v>45225</v>
+      </c>
+      <c r="U25" s="2">
+        <f t="shared" ca="1" si="27"/>
+        <v>26625</v>
+      </c>
+      <c r="V25" s="1">
+        <f t="shared" ca="1" si="27"/>
+        <v>22850</v>
+      </c>
+      <c r="W25" s="2">
+        <f t="shared" ca="1" si="27"/>
+        <v>52375</v>
+      </c>
+      <c r="X25" s="3">
+        <f t="shared" si="27"/>
         <v>709937.5</v>
+      </c>
+      <c r="Y25" s="2">
+        <f t="shared" ca="1" si="27"/>
+        <v>483825</v>
+      </c>
+      <c r="Z25" s="1">
+        <f t="shared" ca="1" si="27"/>
+        <v>411875</v>
+      </c>
+      <c r="AA25" s="2">
+        <f t="shared" ca="1" si="27"/>
+        <v>423300</v>
+      </c>
+      <c r="AB25" s="1">
+        <f t="shared" ca="1" si="27"/>
+        <v>503625</v>
+      </c>
+      <c r="AC25" s="1"/>
+      <c r="AD25" s="1">
+        <f t="shared" ref="AC25:AD25" ca="1" si="28">SUM(AD4:AD20)</f>
+        <v>2532562.5</v>
       </c>
     </row>
   </sheetData>
@@ -1196,5 +3205,6 @@
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="25" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>